<commit_message>
automation of pcb renders
</commit_message>
<xml_diff>
--- a/amulet_controller/Generated/Manufacturing/Assembly/amulet_controller-bom.xlsx
+++ b/amulet_controller/Generated/Manufacturing/Assembly/amulet_controller-bom.xlsx
@@ -1783,7 +1783,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>8.0.5-8.0.5-0~ubuntu24.04.1</t>
+    <t>8.0.6-8.0.6-0~ubuntu24.04.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -1831,7 +1831,7 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2024-11-01 00:44:16</t>
+    <t>2024-11-12 19:29:53</t>
   </si>
   <si>
     <t>KiCost® v1.1.18 + KiBot v1.8.3</t>

</xml_diff>